<commit_message>
Header, Footer, Hero block and Discover tabs block
Automated migration updates generated by Experience Modernization Agent.

Changed files (14):
- blocks/footer/footer.css
- blocks/footer/footer.js
- blocks/hero-event/hero-event.css
- blocks/hero-event/hero-event.js
- blocks/search-form/search-form.css
- blocks/search-form/search-form.js
- blocks/tabs-discovery/tabs-discovery.css
- blocks/tabs-discovery/tabs-discovery.js
- blocks/tabs-discovery/tabs-tokens.css
- footer.plain.html
- tools/importer/reports/default.report.json
- tools/importer/reports/import-marriott-homepage.report.xlsx
- tools/importer/reports/reports.report.xlsx
- tools/importer/run-notarget-import.mjs
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-marriott-homepage.report.xlsx
+++ b/tools/importer/reports/import-marriott-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>default.report.json</t>
   </si>
   <si>
-    <t>["hero-event","cards-promo","tabs-discovery","columns-membership","cards-mini","tabs-brands"]</t>
+    <t>["hero-event","cards-promo","tabs-discovery","card-carousel-offers","columns-membership","card-carousel-rentals","cards-mini","tabs-brands"]</t>
   </si>
   <si>
     <t>default</t>
@@ -52,13 +52,13 @@
     <t>marriott-homepage</t>
   </si>
   <si>
-    <t>2026-04-03T11:48:02.425Z</t>
+    <t>2026-04-14T12:46:51.230Z</t>
   </si>
   <si>
     <t>Marriott Bonvoy Hotels | Book Directly &amp; Get Exclusive Rates</t>
   </si>
   <si>
-    <t>https://www.marriott.com/default.mi</t>
+    <t>https://www.marriott.com/default.mi?mboxDisable=1</t>
   </si>
 </sst>
 </file>
@@ -454,8 +454,7 @@
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="37" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>